<commit_message>
feat(BitRuisseau[WIP]): essais de connexion au bon topic
</commit_message>
<xml_diff>
--- a/doc/T-Jercleuet-BitRuisseau-321.xlsx
+++ b/doc/T-Jercleuet-BitRuisseau-321.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pt04ihk\Documents\GitHub\321-BitRuisseau\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4085C2B9-593A-4388-8525-C0C3E4258E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E1E15B7-97FA-40AF-8B1B-1FECA844CCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="59">
   <si>
     <t>Auteur:</t>
   </si>
@@ -212,6 +212,12 @@
   </si>
   <si>
     <t>Tentatives d'implémentation de la communication avec le protocole</t>
+  </si>
+  <si>
+    <t>Essai infructueux de copier le backend de powercher</t>
+  </si>
+  <si>
+    <t>Copie des fichiers MQTTCommunicator et Icommunicator du backend de powercher et adaptation pour ne plus avoir d'erreurs</t>
   </si>
 </sst>
 </file>
@@ -1329,7 +1335,7 @@
       <c r="B3" s="52"/>
       <c r="C3" s="43" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>14 heures 25 minutes</v>
+        <v>14 heures 55 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -1348,11 +1354,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>505</v>
+        <v>535</v>
       </c>
       <c r="E4" s="21">
         <f>SUM(C4:D4)</f>
-        <v>865</v>
+        <v>895</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -1990,21 +1996,35 @@
         <v>46006</v>
       </c>
       <c r="C34" s="28"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="19"/>
+      <c r="D34" s="29">
+        <v>20</v>
+      </c>
+      <c r="E34" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" s="19" t="s">
+        <v>57</v>
+      </c>
       <c r="G34" s="36"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="40" t="str">
+    <row r="35" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="40">
         <f>IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
-        <v/>
-      </c>
-      <c r="B35" s="31"/>
+        <v>51</v>
+      </c>
+      <c r="B35" s="31">
+        <v>46006</v>
+      </c>
       <c r="C35" s="32"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="20"/>
+      <c r="D35" s="33">
+        <v>10</v>
+      </c>
+      <c r="E35" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" s="20" t="s">
+        <v>58</v>
+      </c>
       <c r="G35" s="37"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -14649,14 +14669,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14861,23 +14879,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -14902,9 +14917,14 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
doc(jdt): update du jdt
</commit_message>
<xml_diff>
--- a/doc/T-Jercleuet-BitRuisseau-321.xlsx
+++ b/doc/T-Jercleuet-BitRuisseau-321.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pt04ihk\Documents\GitHub\321-BitRuisseau\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E1E15B7-97FA-40AF-8B1B-1FECA844CCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A4EA784-BC0B-4014-A0A0-B11F508B970C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="62">
   <si>
     <t>Auteur:</t>
   </si>
@@ -218,6 +218,15 @@
   </si>
   <si>
     <t>Copie des fichiers MQTTCommunicator et Icommunicator du backend de powercher et adaptation pour ne plus avoir d'erreurs</t>
+  </si>
+  <si>
+    <t>Corrections dans le MQTTService pour envoyer les bons messages et corrections dans l'affichage pour afficher les Mediacenter distants</t>
+  </si>
+  <si>
+    <t>Avec le reste de la classe, mise en commun pour que tout le monde puisse se voir sur le réseau</t>
+  </si>
+  <si>
+    <t>Revue du feedback avec le prof + test "loup garou"</t>
   </si>
 </sst>
 </file>
@@ -1335,7 +1344,7 @@
       <c r="B3" s="52"/>
       <c r="C3" s="43" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>14 heures 55 minutes</v>
+        <v>18 heures 55 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -1350,7 +1359,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>360</v>
+        <v>600</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -1358,7 +1367,7 @@
       </c>
       <c r="E4" s="21">
         <f>SUM(C4:D4)</f>
-        <v>895</v>
+        <v>1135</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -2028,39 +2037,63 @@
       <c r="G35" s="37"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="39" t="str">
+      <c r="A36" s="39">
         <f>IF(ISBLANK(B36),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B36))</f>
-        <v/>
-      </c>
-      <c r="B36" s="27"/>
-      <c r="C36" s="28"/>
+        <v>1</v>
+      </c>
+      <c r="B36" s="27">
+        <v>46026</v>
+      </c>
+      <c r="C36" s="28">
+        <v>1</v>
+      </c>
       <c r="D36" s="29"/>
-      <c r="E36" s="30"/>
-      <c r="F36" s="19"/>
+      <c r="E36" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" s="19" t="s">
+        <v>59</v>
+      </c>
       <c r="G36" s="36"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="40" t="str">
+      <c r="A37" s="40">
         <f>IF(ISBLANK(B37),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B37))</f>
-        <v/>
-      </c>
-      <c r="B37" s="31"/>
-      <c r="C37" s="32"/>
+        <v>2</v>
+      </c>
+      <c r="B37" s="31">
+        <v>46027</v>
+      </c>
+      <c r="C37" s="32">
+        <v>2</v>
+      </c>
       <c r="D37" s="33"/>
-      <c r="E37" s="34"/>
-      <c r="F37" s="19"/>
+      <c r="E37" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" s="19" t="s">
+        <v>60</v>
+      </c>
       <c r="G37" s="37"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="39" t="str">
+      <c r="A38" s="39">
         <f>IF(ISBLANK(B38),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B38))</f>
-        <v/>
-      </c>
-      <c r="B38" s="27"/>
-      <c r="C38" s="28"/>
+        <v>2</v>
+      </c>
+      <c r="B38" s="27">
+        <v>46027</v>
+      </c>
+      <c r="C38" s="28">
+        <v>1</v>
+      </c>
       <c r="D38" s="29"/>
-      <c r="E38" s="30"/>
-      <c r="F38" s="19"/>
+      <c r="E38" s="30" t="s">
+        <v>2</v>
+      </c>
+      <c r="F38" s="19" t="s">
+        <v>61</v>
+      </c>
       <c r="G38" s="36"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>